<commit_message>
New final edit of all
</commit_message>
<xml_diff>
--- a/Vlad/export/Приложение_А.xlsx
+++ b/Vlad/export/Приложение_А.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD15"/>
+  <dimension ref="A1:BH15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,10 @@
     <col width="14" customWidth="1" min="54" max="54"/>
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -757,15 +761,35 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>Mw1</t>
+          <t>Mw1вт</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
         <is>
-          <t>Mc2cp</t>
+          <t>Mc2вт</t>
         </is>
       </c>
       <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Mw1ср</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Mc2ср</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Mw1п</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Mc2п</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>d'2</t>
         </is>
@@ -932,12 +956,24 @@
         <v>273.4</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>0.731</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.8017</v>
       </c>
       <c r="BD2" s="2" t="n">
+        <v>0.7309</v>
+      </c>
+      <c r="BE2" s="2" t="n">
+        <v>0.6903</v>
+      </c>
+      <c r="BF2" s="2" t="n">
+        <v>0.6708</v>
+      </c>
+      <c r="BG2" s="2" t="n">
+        <v>0.6415</v>
+      </c>
+      <c r="BH2" s="2" t="n">
         <v>0.5531</v>
       </c>
     </row>
@@ -1102,12 +1138,24 @@
         <v>302.7</v>
       </c>
       <c r="BB3" s="2" t="n">
+        <v>0.7979000000000001</v>
+      </c>
+      <c r="BC3" s="2" t="n">
+        <v>0.7544999999999999</v>
+      </c>
+      <c r="BD3" s="2" t="n">
         <v>0.706</v>
       </c>
-      <c r="BC3" s="2" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="BD3" s="2" t="n">
+      <c r="BE3" s="2" t="n">
+        <v>0.6692</v>
+      </c>
+      <c r="BF3" s="2" t="n">
+        <v>0.6601</v>
+      </c>
+      <c r="BG3" s="2" t="n">
+        <v>0.6324</v>
+      </c>
+      <c r="BH3" s="2" t="n">
         <v>0.6474</v>
       </c>
     </row>
@@ -1272,12 +1320,24 @@
         <v>334.3</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.753</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.651</v>
+        <v>0.7157</v>
       </c>
       <c r="BD4" s="2" t="n">
+        <v>0.6839</v>
+      </c>
+      <c r="BE4" s="2" t="n">
+        <v>0.6509</v>
+      </c>
+      <c r="BF4" s="2" t="n">
+        <v>0.6479</v>
+      </c>
+      <c r="BG4" s="2" t="n">
+        <v>0.6217</v>
+      </c>
+      <c r="BH4" s="2" t="n">
         <v>0.7192</v>
       </c>
     </row>
@@ -1442,12 +1502,24 @@
         <v>367.8</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.655</v>
+        <v>0.7073</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>0.627</v>
+        <v>0.6758</v>
       </c>
       <c r="BD5" s="2" t="n">
+        <v>0.6553</v>
+      </c>
+      <c r="BE5" s="2" t="n">
+        <v>0.6267</v>
+      </c>
+      <c r="BF5" s="2" t="n">
+        <v>0.6263</v>
+      </c>
+      <c r="BG5" s="2" t="n">
+        <v>0.6024</v>
+      </c>
+      <c r="BH5" s="2" t="n">
         <v>0.7714</v>
       </c>
     </row>
@@ -1612,12 +1684,24 @@
         <v>401.5</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>0.629</v>
+        <v>0.67</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>0.604</v>
+        <v>0.6427</v>
       </c>
       <c r="BD6" s="2" t="n">
+        <v>0.6294999999999999</v>
+      </c>
+      <c r="BE6" s="2" t="n">
+        <v>0.6042</v>
+      </c>
+      <c r="BF6" s="2" t="n">
+        <v>0.6057</v>
+      </c>
+      <c r="BG6" s="2" t="n">
+        <v>0.5836</v>
+      </c>
+      <c r="BH6" s="2" t="n">
         <v>0.8095</v>
       </c>
     </row>
@@ -1782,12 +1866,24 @@
         <v>435.3</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>0.606</v>
+        <v>0.6387</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>0.583</v>
+        <v>0.6143</v>
       </c>
       <c r="BD7" s="2" t="n">
+        <v>0.6062</v>
+      </c>
+      <c r="BE7" s="2" t="n">
+        <v>0.5835</v>
+      </c>
+      <c r="BF7" s="2" t="n">
+        <v>0.5863</v>
+      </c>
+      <c r="BG7" s="2" t="n">
+        <v>0.5659</v>
+      </c>
+      <c r="BH7" s="2" t="n">
         <v>0.8384</v>
       </c>
     </row>
@@ -1952,12 +2048,24 @@
         <v>469.2</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>0.585</v>
+        <v>0.6116</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.5896</v>
       </c>
       <c r="BD8" s="2" t="n">
+        <v>0.5851</v>
+      </c>
+      <c r="BE8" s="2" t="n">
+        <v>0.5644</v>
+      </c>
+      <c r="BF8" s="2" t="n">
+        <v>0.5683</v>
+      </c>
+      <c r="BG8" s="2" t="n">
+        <v>0.5492</v>
+      </c>
+      <c r="BH8" s="2" t="n">
         <v>0.8608</v>
       </c>
     </row>
@@ -2122,12 +2230,24 @@
         <v>503</v>
       </c>
       <c r="BB9" s="2" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="BC9" s="2" t="n">
+        <v>0.5678</v>
+      </c>
+      <c r="BD9" s="2" t="n">
         <v>0.5659999999999999</v>
       </c>
-      <c r="BC9" s="2" t="n">
-        <v>0.547</v>
-      </c>
-      <c r="BD9" s="2" t="n">
+      <c r="BE9" s="2" t="n">
+        <v>0.5468</v>
+      </c>
+      <c r="BF9" s="2" t="n">
+        <v>0.5515</v>
+      </c>
+      <c r="BG9" s="2" t="n">
+        <v>0.5336</v>
+      </c>
+      <c r="BH9" s="2" t="n">
         <v>0.8786</v>
       </c>
     </row>
@@ -2292,12 +2412,24 @@
         <v>536.7</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>0.549</v>
+        <v>0.5671</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>0.531</v>
+        <v>0.5484</v>
       </c>
       <c r="BD10" s="2" t="n">
+        <v>0.5485</v>
+      </c>
+      <c r="BE10" s="2" t="n">
+        <v>0.5306999999999999</v>
+      </c>
+      <c r="BF10" s="2" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="BG10" s="2" t="n">
+        <v>0.519</v>
+      </c>
+      <c r="BH10" s="2" t="n">
         <v>0.893</v>
       </c>
     </row>
@@ -2462,12 +2594,24 @@
         <v>570.3</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>0.533</v>
+        <v>0.5484</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>0.516</v>
+        <v>0.5309</v>
       </c>
       <c r="BD11" s="2" t="n">
+        <v>0.5326</v>
+      </c>
+      <c r="BE11" s="2" t="n">
+        <v>0.5158</v>
+      </c>
+      <c r="BF11" s="2" t="n">
+        <v>0.5216</v>
+      </c>
+      <c r="BG11" s="2" t="n">
+        <v>0.5054</v>
+      </c>
+      <c r="BH11" s="2" t="n">
         <v>0.9048</v>
       </c>
     </row>
@@ -2632,12 +2776,24 @@
         <v>603.7</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>0.518</v>
+        <v>0.5316</v>
       </c>
       <c r="BC12" s="2" t="n">
+        <v>0.5151</v>
+      </c>
+      <c r="BD12" s="2" t="n">
+        <v>0.5179</v>
+      </c>
+      <c r="BE12" s="2" t="n">
         <v>0.502</v>
       </c>
-      <c r="BD12" s="2" t="n">
+      <c r="BF12" s="2" t="n">
+        <v>0.5082</v>
+      </c>
+      <c r="BG12" s="2" t="n">
+        <v>0.4928</v>
+      </c>
+      <c r="BH12" s="2" t="n">
         <v>0.9147</v>
       </c>
     </row>
@@ -2802,12 +2958,24 @@
         <v>637</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>0.504</v>
+        <v>0.5131</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>0.489</v>
+        <v>0.4983</v>
       </c>
       <c r="BD13" s="2" t="n">
+        <v>0.5044</v>
+      </c>
+      <c r="BE13" s="2" t="n">
+        <v>0.4893</v>
+      </c>
+      <c r="BF13" s="2" t="n">
+        <v>0.4924</v>
+      </c>
+      <c r="BG13" s="2" t="n">
+        <v>0.4785</v>
+      </c>
+      <c r="BH13" s="2" t="n">
         <v>0.9224</v>
       </c>
     </row>
@@ -2972,12 +3140,24 @@
         <v>670.6</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>0.494</v>
+        <v>0.5016</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>0.458</v>
+        <v>0.467</v>
       </c>
       <c r="BD14" s="2" t="n">
+        <v>0.4943</v>
+      </c>
+      <c r="BE14" s="2" t="n">
+        <v>0.4579</v>
+      </c>
+      <c r="BF14" s="2" t="n">
+        <v>0.4873</v>
+      </c>
+      <c r="BG14" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BH14" s="2" t="n">
         <v>0.9282</v>
       </c>
     </row>
@@ -3142,12 +3322,24 @@
         <v>702.6</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>0.492</v>
+        <v>0.4975</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>0.424</v>
+        <v>0.4334</v>
       </c>
       <c r="BD15" s="2" t="n">
+        <v>0.4917</v>
+      </c>
+      <c r="BE15" s="2" t="n">
+        <v>0.4239</v>
+      </c>
+      <c r="BF15" s="2" t="n">
+        <v>0.4899</v>
+      </c>
+      <c r="BG15" s="2" t="n">
+        <v>0.4188</v>
+      </c>
+      <c r="BH15" s="2" t="n">
         <v>0.9313</v>
       </c>
     </row>

</xml_diff>